<commit_message>
minor updates (sign digits)
</commit_message>
<xml_diff>
--- a/curation/draft/package16/R16_BC_Misc_Edits.xlsx
+++ b/curation/draft/package16/R16_BC_Misc_Edits.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\_github\cdisc-org\COSMoS\curation\draft\package16\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56478847-0763-4065-A98B-1ED66981748F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9415D449-271D-4EAF-8263-A06861038F65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{F590C486-C613-40E0-BF06-47BB8CB37E44}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="45">
   <si>
     <t>package_date</t>
   </si>
@@ -162,6 +162,15 @@
   </si>
   <si>
     <t>datetime</t>
+  </si>
+  <si>
+    <t>Characteristic</t>
+  </si>
+  <si>
+    <t>C25447</t>
+  </si>
+  <si>
+    <t>The distinguishing qualities or prominent aspect of a person, object, action, process, or substance.</t>
   </si>
 </sst>
 </file>
@@ -976,8 +985,28 @@
       </c>
       <c r="Q7" s="4"/>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A8" s="3"/>
+    <row r="8" spans="1:17" ht="45" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="E8" s="6"/>
+      <c r="F8" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="4" t="s">
+        <v>44</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
@@ -996,12 +1025,34 @@
     <hyperlink ref="N7" r:id="rId12" xr:uid="{EDF7ACA4-CAAF-47F7-9EE9-98524ED83205}"/>
     <hyperlink ref="E2" r:id="rId13" display="https://evsexplore.semantics.cancer.gov/evsexplore/concept/ncit/C171083" xr:uid="{BB8BD445-12F9-478C-8721-D0045EF8DDCF}"/>
     <hyperlink ref="E3:E7" r:id="rId14" display="https://evsexplore.semantics.cancer.gov/evsexplore/concept/ncit/C171083" xr:uid="{655D8606-E6F9-47A8-9220-A6087E3333DB}"/>
+    <hyperlink ref="D8" r:id="rId15" xr:uid="{52BEFAFF-714C-4196-BF97-1EBF0BCB1278}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Description0 xmlns="3dc215b4-4765-4137-95ef-e24fb8216673">Data and Metadata documentation will explain structure and content any QC manipulations that have been done to the data.</Description0>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3dc215b4-4765-4137-95ef-e24fb8216673">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2634c873-c79e-4fdd-b8bf-a33e5fa5c27f" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EA3DD6FD0640724CAC6A104AA4040E53" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="866aaee467307fab2f51bbdbaaea79d8">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3dc215b4-4765-4137-95ef-e24fb8216673" xmlns:ns3="2634c873-c79e-4fdd-b8bf-a33e5fa5c27f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="636a025d234e12dfc0e20f1263040641" ns2:_="" ns3:_="">
     <xsd:import namespace="3dc215b4-4765-4137-95ef-e24fb8216673"/>
@@ -1258,28 +1309,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Description0 xmlns="3dc215b4-4765-4137-95ef-e24fb8216673">Data and Metadata documentation will explain structure and content any QC manipulations that have been done to the data.</Description0>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3dc215b4-4765-4137-95ef-e24fb8216673">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2634c873-c79e-4fdd-b8bf-a33e5fa5c27f" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{54257E14-FF77-411D-9C84-0AB47C32F166}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F20F3C00-18F9-4A8E-8FC6-0E813A118EF8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="3dc215b4-4765-4137-95ef-e24fb8216673"/>
+    <ds:schemaRef ds:uri="2634c873-c79e-4fdd-b8bf-a33e5fa5c27f"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9BBDDA1-B2C2-48AC-A803-F46C63765243}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1296,23 +1345,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F20F3C00-18F9-4A8E-8FC6-0E813A118EF8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="3dc215b4-4765-4137-95ef-e24fb8216673"/>
-    <ds:schemaRef ds:uri="2634c873-c79e-4fdd-b8bf-a33e5fa5c27f"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{54257E14-FF77-411D-9C84-0AB47C32F166}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>